<commit_message>
Fix reconciliation, recovery exports and native document failures
</commit_message>
<xml_diff>
--- a/examples/catl-2025/deliverables/workbook.xlsx
+++ b/examples/catl-2025/deliverables/workbook.xlsx
@@ -24,16 +24,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Findings!$A$1:$I$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Procedures!$A$1:$J$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Readme!$A$1:$B$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Reconciliations!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Reconciliations!$A$1:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Requests!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sources!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sources!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1656" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1658" uniqueCount="514">
   <si>
     <t>字段 / field</t>
   </si>
@@ -1094,13 +1094,16 @@
     <t>容差依据</t>
   </si>
   <si>
+    <t>未测试原因</t>
+  </si>
+  <si>
     <t>R_BS</t>
   </si>
   <si>
     <t>资产负债关系</t>
   </si>
   <si>
-    <t>within_precision</t>
+    <t>within_input_tolerance</t>
   </si>
   <si>
     <t>基础单位人民币；原表以千元披露。按参加计算项目的独立舍入上界保留残差，不将容差内残差强制归零。</t>
@@ -1170,6 +1173,9 @@
   </si>
   <si>
     <t>SHA256</t>
+  </si>
+  <si>
+    <t>时间证据与限制</t>
   </si>
   <si>
     <t>AR</t>
@@ -2127,7 +2133,7 @@
         <v>1000</v>
       </c>
       <c r="F2" s="3">
-        <f>D2*E2</f>
+        <f>IF(COUNT(D2,E2)=2,D2*E2,NA())</f>
         <v>423701834000.0</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -2180,7 +2186,7 @@
         <v>1000</v>
       </c>
       <c r="F3" s="3">
-        <f>D3*E3</f>
+        <f>IF(COUNT(D3,E3)=2,D3*E3,NA())</f>
         <v>362012554000.0</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -2233,7 +2239,7 @@
         <v>1000</v>
       </c>
       <c r="F4" s="3">
-        <f>D4*E4</f>
+        <f>IF(COUNT(D4,E4)=2,D4*E4,NA())</f>
         <v>312383297000.0</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -2286,7 +2292,7 @@
         <v>1000</v>
       </c>
       <c r="F5" s="3">
-        <f>D5*E5</f>
+        <f>IF(COUNT(D5,E5)=2,D5*E5,NA())</f>
         <v>273518959000.0</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -2339,7 +2345,7 @@
         <v>1000</v>
       </c>
       <c r="F6" s="3">
-        <f>D6*E6</f>
+        <f>IF(COUNT(D6,E6)=2,D6*E6,NA())</f>
         <v>76786309000.0</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -2392,7 +2398,7 @@
         <v>1000</v>
       </c>
       <c r="F7" s="3">
-        <f>D7*E7</f>
+        <f>IF(COUNT(D7,E7)=2,D7*E7,NA())</f>
         <v>54006794000.0</v>
       </c>
       <c r="G7" s="2" t="s">
@@ -2445,7 +2451,7 @@
         <v>1000</v>
       </c>
       <c r="F8" s="3">
-        <f>D8*E8</f>
+        <f>IF(COUNT(D8,E8)=2,D8*E8,NA())</f>
         <v>133219982000.0</v>
       </c>
       <c r="G8" s="2" t="s">
@@ -2498,7 +2504,7 @@
         <v>1000</v>
       </c>
       <c r="F9" s="3">
-        <f>D9*E9</f>
+        <f>IF(COUNT(D9,E9)=2,D9*E9,NA())</f>
         <v>96990345000.0</v>
       </c>
       <c r="G9" s="2" t="s">
@@ -2551,7 +2557,7 @@
         <v>1000</v>
       </c>
       <c r="F10" s="3">
-        <f>D10*E10</f>
+        <f>IF(COUNT(D10,E10)=2,D10*E10,NA())</f>
         <v>299929741000.0</v>
       </c>
       <c r="G10" s="2" t="s">
@@ -2602,7 +2608,7 @@
         <v>1000</v>
       </c>
       <c r="F11" s="3">
-        <f>D11*E11</f>
+        <f>IF(COUNT(D11,E11)=2,D11*E11,NA())</f>
         <v>270159734000.0</v>
       </c>
       <c r="G11" s="2" t="s">
@@ -2653,7 +2659,7 @@
         <v>1000</v>
       </c>
       <c r="F12" s="3">
-        <f>D12*E12</f>
+        <f>IF(COUNT(D12,E12)=2,D12*E12,NA())</f>
         <v>974827544000.0</v>
       </c>
       <c r="G12" s="2" t="s">
@@ -2704,7 +2710,7 @@
         <v>1000</v>
       </c>
       <c r="F13" s="3">
-        <f>D13*E13</f>
+        <f>IF(COUNT(D13,E13)=2,D13*E13,NA())</f>
         <v>786658123000.0</v>
       </c>
       <c r="G13" s="2" t="s">
@@ -2755,7 +2761,7 @@
         <v>1000</v>
       </c>
       <c r="F14" s="3">
-        <f>D14*E14</f>
+        <f>IF(COUNT(D14,E14)=2,D14*E14,NA())</f>
         <v>371026324000.0</v>
       </c>
       <c r="G14" s="2" t="s">
@@ -2806,7 +2812,7 @@
         <v>1000</v>
       </c>
       <c r="F15" s="3">
-        <f>D15*E15</f>
+        <f>IF(COUNT(D15,E15)=2,D15*E15,NA())</f>
         <v>273456174000.0</v>
       </c>
       <c r="G15" s="2" t="s">
@@ -2857,7 +2863,7 @@
         <v>1000</v>
       </c>
       <c r="F16" s="3">
-        <f>D16*E16</f>
+        <f>IF(COUNT(D16,E16)=2,D16*E16,NA())</f>
         <v>337107747000.0</v>
       </c>
       <c r="G16" s="2" t="s">
@@ -2908,7 +2914,7 @@
         <v>1000</v>
       </c>
       <c r="F17" s="3">
-        <f>D17*E17</f>
+        <f>IF(COUNT(D17,E17)=2,D17*E17,NA())</f>
         <v>246930033000.0</v>
       </c>
       <c r="G17" s="2" t="s">
@@ -2959,7 +2965,7 @@
         <v>1000</v>
       </c>
       <c r="F18" s="3">
-        <f>D18*E18</f>
+        <f>IF(COUNT(D18,E18)=2,D18*E18,NA())</f>
         <v>94526239000.0</v>
       </c>
       <c r="G18" s="2" t="s">
@@ -3010,7 +3016,7 @@
         <v>1000</v>
       </c>
       <c r="F19" s="3">
-        <f>D19*E19</f>
+        <f>IF(COUNT(D19,E19)=2,D19*E19,NA())</f>
         <v>59835533000.0</v>
       </c>
       <c r="G19" s="2" t="s">
@@ -3061,7 +3067,7 @@
         <v>1000</v>
       </c>
       <c r="F20" s="3">
-        <f>D20*E20</f>
+        <f>IF(COUNT(D20,E20)=2,D20*E20,NA())</f>
         <v>76403264000.0</v>
       </c>
       <c r="G20" s="2" t="s">
@@ -3112,7 +3118,7 @@
         <v>1000</v>
       </c>
       <c r="F21" s="3">
-        <f>D21*E21</f>
+        <f>IF(COUNT(D21,E21)=2,D21*E21,NA())</f>
         <v>64135510000.0</v>
       </c>
       <c r="G21" s="2" t="s">
@@ -3163,7 +3169,7 @@
         <v>1000</v>
       </c>
       <c r="F22" s="3">
-        <f>D22*E22</f>
+        <f>IF(COUNT(D22,E22)=2,D22*E22,NA())</f>
         <v>160328962000.0</v>
       </c>
       <c r="G22" s="2" t="s">
@@ -3214,7 +3220,7 @@
         <v>1000</v>
       </c>
       <c r="F23" s="3">
-        <f>D23*E23</f>
+        <f>IF(COUNT(D23,E23)=2,D23*E23,NA())</f>
         <v>130977408000.0</v>
       </c>
       <c r="G23" s="2" t="s">
@@ -3265,7 +3271,7 @@
         <v>1000</v>
       </c>
       <c r="F24" s="3">
-        <f>D24*E24</f>
+        <f>IF(COUNT(D24,E24)=2,D24*E24,NA())</f>
         <v>49233377000.0</v>
       </c>
       <c r="G24" s="2" t="s">
@@ -3316,7 +3322,7 @@
         <v>1000</v>
       </c>
       <c r="F25" s="3">
-        <f>D25*E25</f>
+        <f>IF(COUNT(D25,E25)=2,D25*E25,NA())</f>
         <v>27834446000.0</v>
       </c>
       <c r="G25" s="2" t="s">
@@ -3367,7 +3373,7 @@
         <v>1000</v>
       </c>
       <c r="F26" s="3">
-        <f>D26*E26</f>
+        <f>IF(COUNT(D26,E26)=2,D26*E26,NA())</f>
         <v>37222781000.0</v>
       </c>
       <c r="G26" s="2" t="s">
@@ -3418,7 +3424,7 @@
         <v>1000</v>
       </c>
       <c r="F27" s="3">
-        <f>D27*E27</f>
+        <f>IF(COUNT(D27,E27)=2,D27*E27,NA())</f>
         <v>44362409000.0</v>
       </c>
       <c r="G27" s="2" t="s">
@@ -3469,7 +3475,7 @@
         <v>1000</v>
       </c>
       <c r="F28" s="3">
-        <f>D28*E28</f>
+        <f>IF(COUNT(D28,E28)=2,D28*E28,NA())</f>
         <v>51233080000.0</v>
       </c>
       <c r="G28" s="2" t="s">
@@ -3520,7 +3526,7 @@
         <v>1000</v>
       </c>
       <c r="F29" s="3">
-        <f>D29*E29</f>
+        <f>IF(COUNT(D29,E29)=2,D29*E29,NA())</f>
         <v>39070181000.0</v>
       </c>
       <c r="G29" s="2" t="s">
@@ -3571,7 +3577,7 @@
         <v>1000</v>
       </c>
       <c r="F30" s="3">
-        <f>D30*E30</f>
+        <f>IF(COUNT(D30,E30)=2,D30*E30,NA())</f>
         <v>119601197000.0</v>
       </c>
       <c r="G30" s="2" t="s">
@@ -3622,7 +3628,7 @@
         <v>1000</v>
       </c>
       <c r="F31" s="3">
-        <f>D31*E31</f>
+        <f>IF(COUNT(D31,E31)=2,D31*E31,NA())</f>
         <v>136346553000.0</v>
       </c>
       <c r="G31" s="2" t="s">
@@ -3673,7 +3679,7 @@
         <v>1000</v>
       </c>
       <c r="F32" s="3">
-        <f>D32*E32</f>
+        <f>IF(COUNT(D32,E32)=2,D32*E32,NA())</f>
         <v>316506369000.0</v>
       </c>
       <c r="G32" s="2" t="s">
@@ -3726,7 +3732,7 @@
         <v>1000</v>
       </c>
       <c r="F33" s="3">
-        <f>D33*E33</f>
+        <f>IF(COUNT(D33,E33)=2,D33*E33,NA())</f>
         <v>253041337000.0</v>
       </c>
       <c r="G33" s="2" t="s">
@@ -3779,7 +3785,7 @@
         <v>1000</v>
       </c>
       <c r="F34" s="3">
-        <f>D34*E34</f>
+        <f>IF(COUNT(D34,E34)=2,D34*E34,NA())</f>
         <v>62439820000.0</v>
       </c>
       <c r="G34" s="2" t="s">
@@ -3832,7 +3838,7 @@
         <v>1000</v>
       </c>
       <c r="F35" s="3">
-        <f>D35*E35</f>
+        <f>IF(COUNT(D35,E35)=2,D35*E35,NA())</f>
         <v>57290460000.0</v>
       </c>
       <c r="G35" s="2" t="s">
@@ -3885,7 +3891,7 @@
         <v>1000</v>
       </c>
       <c r="F36" s="3">
-        <f>D36*E36</f>
+        <f>IF(COUNT(D36,E36)=2,D36*E36,NA())</f>
         <v>21860936000.0</v>
       </c>
       <c r="G36" s="2" t="s">
@@ -3938,7 +3944,7 @@
         <v>1000</v>
       </c>
       <c r="F37" s="3">
-        <f>D37*E37</f>
+        <f>IF(COUNT(D37,E37)=2,D37*E37,NA())</f>
         <v>28699935000.0</v>
       </c>
       <c r="G37" s="2" t="s">
@@ -3991,7 +3997,7 @@
         <v>1000</v>
       </c>
       <c r="F38" s="3">
-        <f>D38*E38</f>
+        <f>IF(COUNT(D38,E38)=2,D38*E38,NA())</f>
         <v>72201282000.0</v>
       </c>
       <c r="G38" s="2" t="s">
@@ -4044,7 +4050,7 @@
         <v>1000</v>
       </c>
       <c r="F39" s="3">
-        <f>D39*E39</f>
+        <f>IF(COUNT(D39,E39)=2,D39*E39,NA())</f>
         <v>4585027000.0</v>
       </c>
       <c r="G39" s="2" t="s">
@@ -4097,7 +4103,7 @@
         <v>1000</v>
       </c>
       <c r="F40" s="3">
-        <f>D40*E40</f>
+        <f>IF(COUNT(D40,E40)=2,D40*E40,NA())</f>
         <v>-94475790000.0</v>
       </c>
       <c r="G40" s="2" t="s">
@@ -4150,7 +4156,7 @@
         <v>1000</v>
       </c>
       <c r="F41" s="3">
-        <f>D41*E41</f>
+        <f>IF(COUNT(D41,E41)=2,D41*E41,NA())</f>
         <v>-6309543000.0</v>
       </c>
       <c r="G41" s="2" t="s">
@@ -4203,7 +4209,7 @@
         <v>1000</v>
       </c>
       <c r="F42" s="3">
-        <f>D42*E42</f>
+        <f>IF(COUNT(D42,E42)=2,D42*E42,NA())</f>
         <v>-2664640000.0</v>
       </c>
       <c r="G42" s="2" t="s">
@@ -4256,7 +4262,7 @@
         <v>1000</v>
       </c>
       <c r="F43" s="3">
-        <f>D43*E43</f>
+        <f>IF(COUNT(D43,E43)=2,D43*E43,NA())</f>
         <v>29770008000.0</v>
       </c>
       <c r="G43" s="2" t="s">
@@ -4309,7 +4315,7 @@
         <v>1000</v>
       </c>
       <c r="F44" s="3">
-        <f>D44*E44</f>
+        <f>IF(COUNT(D44,E44)=2,D44*E44,NA())</f>
         <v>42344558000.0</v>
       </c>
       <c r="G44" s="2" t="s">
@@ -4362,7 +4368,7 @@
         <v>1000</v>
       </c>
       <c r="F45" s="3">
-        <f>D45*E45</f>
+        <f>IF(COUNT(D45,E45)=2,D45*E45,NA())</f>
         <v>84006523000.0</v>
       </c>
       <c r="G45" s="2" t="s">
@@ -4415,7 +4421,7 @@
         <v>1000</v>
       </c>
       <c r="F46" s="3">
-        <f>D46*E46</f>
+        <f>IF(COUNT(D46,E46)=2,D46*E46,NA())</f>
         <v>40416391000.0</v>
       </c>
       <c r="G46" s="2" t="s">
@@ -4468,7 +4474,7 @@
         <v>1000</v>
       </c>
       <c r="F47" s="3">
-        <f>D47*E47</f>
+        <f>IF(COUNT(D47,E47)=2,D47*E47,NA())</f>
         <v>-26842954000.0</v>
       </c>
       <c r="G47" s="2" t="s">
@@ -4521,7 +4527,7 @@
         <v>1000</v>
       </c>
       <c r="F48" s="3">
-        <f>D48*E48</f>
+        <f>IF(COUNT(D48,E48)=2,D48*E48,NA())</f>
         <v>-9811000.0</v>
       </c>
       <c r="G48" s="2" t="s">
@@ -4574,7 +4580,7 @@
         <v>1000</v>
       </c>
       <c r="F49" s="3">
-        <f>D49*E49</f>
+        <f>IF(COUNT(D49,E49)=2,D49*E49,NA())</f>
         <v>39790079000.0</v>
       </c>
       <c r="G49" s="2" t="s">
@@ -4627,7 +4633,7 @@
         <v>1000</v>
       </c>
       <c r="F50" s="3">
-        <f>D50*E50</f>
+        <f>IF(COUNT(D50,E50)=2,D50*E50,NA())</f>
         <v>-54608510000.0</v>
       </c>
       <c r="G50" s="2" t="s">
@@ -4680,7 +4686,7 @@
         <v>1000</v>
       </c>
       <c r="F51" s="3">
-        <f>D51*E51</f>
+        <f>IF(COUNT(D51,E51)=2,D51*E51,NA())</f>
         <v>-1926925000.0</v>
       </c>
       <c r="G51" s="2" t="s">
@@ -4733,7 +4739,7 @@
         <v>1000</v>
       </c>
       <c r="F52" s="3">
-        <f>D52*E52</f>
+        <f>IF(COUNT(D52,E52)=2,D52*E52,NA())</f>
         <v>2659992000.0</v>
       </c>
       <c r="G52" s="2" t="s">
@@ -4786,7 +4792,7 @@
         <v>1000</v>
       </c>
       <c r="F53" s="3">
-        <f>D53*E53</f>
+        <f>IF(COUNT(D53,E53)=2,D53*E53,NA())</f>
         <v>60616240000.0</v>
       </c>
       <c r="G53" s="2" t="s">
@@ -4839,7 +4845,7 @@
         <v>1000</v>
       </c>
       <c r="F54" s="3">
-        <f>D54*E54</f>
+        <f>IF(COUNT(D54,E54)=2,D54*E54,NA())</f>
         <v>603801220000.0</v>
       </c>
       <c r="G54" s="2" t="s">
@@ -4890,7 +4896,7 @@
         <v>1000</v>
       </c>
       <c r="F55" s="3">
-        <f>D55*E55</f>
+        <f>IF(COUNT(D55,E55)=2,D55*E55,NA())</f>
         <v>333512927000.0</v>
       </c>
       <c r="G55" s="2" t="s">
@@ -4941,7 +4947,7 @@
         <v>1000</v>
       </c>
       <c r="F56" s="3">
-        <f>D56*E56</f>
+        <f>IF(COUNT(D56,E56)=2,D56*E56,NA())</f>
         <v>33583185000.0</v>
       </c>
       <c r="G56" s="2" t="s">
@@ -4992,7 +4998,7 @@
         <v>1000</v>
       </c>
       <c r="F57" s="3">
-        <f>D57*E57</f>
+        <f>IF(COUNT(D57,E57)=2,D57*E57,NA())</f>
         <v>18428631000.0</v>
       </c>
       <c r="G57" s="2" t="s">
@@ -5043,7 +5049,7 @@
         <v>1000</v>
       </c>
       <c r="F58" s="3">
-        <f>D58*E58</f>
+        <f>IF(COUNT(D58,E58)=2,D58*E58,NA())</f>
         <v>461587000.0</v>
       </c>
       <c r="G58" s="2" t="s">
@@ -5094,7 +5100,7 @@
         <v>1000</v>
       </c>
       <c r="F59" s="3">
-        <f>D59*E59</f>
+        <f>IF(COUNT(D59,E59)=2,D59*E59,NA())</f>
         <v>14692968000.0</v>
       </c>
       <c r="G59" s="2" t="s">
@@ -5145,7 +5151,7 @@
         <v>1000</v>
       </c>
       <c r="F60" s="3">
-        <f>D60*E60</f>
+        <f>IF(COUNT(D60,E60)=2,D60*E60,NA())</f>
         <v>23902653000.0</v>
       </c>
       <c r="G60" s="2" t="s">
@@ -5196,7 +5202,7 @@
         <v>1000</v>
       </c>
       <c r="F61" s="3">
-        <f>D61*E61</f>
+        <f>IF(COUNT(D61,E61)=2,D61*E61,NA())</f>
         <v>13320128000.0</v>
       </c>
       <c r="G61" s="2" t="s">
@@ -5247,7 +5253,7 @@
         <v>1000</v>
       </c>
       <c r="F62" s="3">
-        <f>D62*E62</f>
+        <f>IF(COUNT(D62,E62)=2,D62*E62,NA())</f>
         <v>30728127000.0</v>
       </c>
       <c r="G62" s="2" t="s">
@@ -5298,7 +5304,7 @@
         <v>1000</v>
       </c>
       <c r="F63" s="3">
-        <f>D63*E63</f>
+        <f>IF(COUNT(D63,E63)=2,D63*E63,NA())</f>
         <v>2865508000.0</v>
       </c>
       <c r="G63" s="2" t="s">
@@ -5349,7 +5355,7 @@
         <v>1000</v>
       </c>
       <c r="F64" s="3">
-        <f>D64*E64</f>
+        <f>IF(COUNT(D64,E64)=2,D64*E64,NA())</f>
         <v>205516000.0</v>
       </c>
       <c r="G64" s="2" t="s">
@@ -5400,7 +5406,7 @@
         <v>1000</v>
       </c>
       <c r="F65" s="3">
-        <f>D65*E65</f>
+        <f>IF(COUNT(D65,E65)=2,D65*E65,NA())</f>
         <v>70414214000.0</v>
       </c>
       <c r="G65" s="2" t="s">
@@ -5453,7 +5459,7 @@
         <v>1</v>
       </c>
       <c r="F66" s="3">
-        <f>D66*E66</f>
+        <f>IF(COUNT(D66,E66)=2,D66*E66,NA())</f>
         <v>661.0</v>
       </c>
       <c r="G66" s="2" t="s">
@@ -5506,7 +5512,7 @@
         <v>1</v>
       </c>
       <c r="F67" s="3">
-        <f>D67*E67</f>
+        <f>IF(COUNT(D67,E67)=2,D67*E67,NA())</f>
         <v>475.0</v>
       </c>
       <c r="G67" s="2" t="s">
@@ -5559,7 +5565,7 @@
         <v>1000</v>
       </c>
       <c r="F68" s="3">
-        <f>D68*E68</f>
+        <f>IF(COUNT(D68,E68)=2,D68*E68,NA())</f>
         <v>8660164000.0</v>
       </c>
       <c r="G68" s="2" t="s">
@@ -5612,7 +5618,7 @@
         <v>1000</v>
       </c>
       <c r="F69" s="3">
-        <f>D69*E69</f>
+        <f>IF(COUNT(D69,E69)=2,D69*E69,NA())</f>
         <v>418585000.0</v>
       </c>
       <c r="G69" s="2" t="s">
@@ -5665,7 +5671,7 @@
         <v>1000</v>
       </c>
       <c r="F70" s="3">
-        <f>D70*E70</f>
+        <f>IF(COUNT(D70,E70)=2,D70*E70,NA())</f>
         <v>24322780000.0</v>
       </c>
       <c r="G70" s="2" t="s">
@@ -5718,7 +5724,7 @@
         <v>1000</v>
       </c>
       <c r="F71" s="3">
-        <f>D71*E71</f>
+        <f>IF(COUNT(D71,E71)=2,D71*E71,NA())</f>
         <v>337367000.0</v>
       </c>
       <c r="G71" s="2" t="s">
@@ -5771,7 +5777,7 @@
         <v>1000</v>
       </c>
       <c r="F72" s="3">
-        <f>D72*E72</f>
+        <f>IF(COUNT(D72,E72)=2,D72*E72,NA())</f>
         <v>512000000.0</v>
       </c>
       <c r="G72" s="2" t="s">
@@ -5824,7 +5830,7 @@
         <v>1000</v>
       </c>
       <c r="F73" s="3">
-        <f>D73*E73</f>
+        <f>IF(COUNT(D73,E73)=2,D73*E73,NA())</f>
         <v>1764508000.0</v>
       </c>
       <c r="G73" s="2" t="s">
@@ -5877,7 +5883,7 @@
         <v>1000</v>
       </c>
       <c r="F74" s="3">
-        <f>D74*E74</f>
+        <f>IF(COUNT(D74,E74)=2,D74*E74,NA())</f>
         <v>-174640000.0</v>
       </c>
       <c r="G74" s="2" t="s">
@@ -5930,7 +5936,7 @@
         <v>1000</v>
       </c>
       <c r="F75" s="3">
-        <f>D75*E75</f>
+        <f>IF(COUNT(D75,E75)=2,D75*E75,NA())</f>
         <v>151291000.0</v>
       </c>
       <c r="G75" s="2" t="s">
@@ -5983,7 +5989,7 @@
         <v>1000</v>
       </c>
       <c r="F76" s="3">
-        <f>D76*E76</f>
+        <f>IF(COUNT(D76,E76)=2,D76*E76,NA())</f>
         <v>-974079000.0</v>
       </c>
       <c r="G76" s="2" t="s">
@@ -6036,7 +6042,7 @@
         <v>1000</v>
       </c>
       <c r="F77" s="3">
-        <f>D77*E77</f>
+        <f>IF(COUNT(D77,E77)=2,D77*E77,NA())</f>
         <v>2470751000.0</v>
       </c>
       <c r="G77" s="2" t="s">
@@ -6089,7 +6095,7 @@
         <v>1000</v>
       </c>
       <c r="F78" s="3">
-        <f>D78*E78</f>
+        <f>IF(COUNT(D78,E78)=2,D78*E78,NA())</f>
         <v>-8429599000.0</v>
       </c>
       <c r="G78" s="2" t="s">
@@ -6142,7 +6148,7 @@
         <v>1000</v>
       </c>
       <c r="F79" s="3">
-        <f>D79*E79</f>
+        <f>IF(COUNT(D79,E79)=2,D79*E79,NA())</f>
         <v>-7660090000.0</v>
       </c>
       <c r="G79" s="2" t="s">
@@ -6195,7 +6201,7 @@
         <v>1000</v>
       </c>
       <c r="F80" s="3">
-        <f>D80*E80</f>
+        <f>IF(COUNT(D80,E80)=2,D80*E80,NA())</f>
         <v>1900952000.0</v>
       </c>
       <c r="G80" s="2" t="s">
@@ -6248,7 +6254,7 @@
         <v>1000</v>
       </c>
       <c r="F81" s="3">
-        <f>D81*E81</f>
+        <f>IF(COUNT(D81,E81)=2,D81*E81,NA())</f>
         <v>-39837988000.0</v>
       </c>
       <c r="G81" s="2" t="s">
@@ -6301,7 +6307,7 @@
         <v>1000</v>
       </c>
       <c r="F82" s="3">
-        <f>D82*E82</f>
+        <f>IF(COUNT(D82,E82)=2,D82*E82,NA())</f>
         <v>-16911542000.0</v>
       </c>
       <c r="G82" s="2" t="s">
@@ -6354,7 +6360,7 @@
         <v>1000</v>
       </c>
       <c r="F83" s="3">
-        <f>D83*E83</f>
+        <f>IF(COUNT(D83,E83)=2,D83*E83,NA())</f>
         <v>89965735000.0</v>
       </c>
       <c r="G83" s="2" t="s">
@@ -6407,7 +6413,7 @@
         <v>1000</v>
       </c>
       <c r="F84" s="3">
-        <f>D84*E84</f>
+        <f>IF(COUNT(D84,E84)=2,D84*E84,NA())</f>
         <v>-82524000.0</v>
       </c>
       <c r="G84" s="2" t="s">
@@ -6522,10 +6528,14 @@
         <f>D2/K2</f>
         <v>111318537.0</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G2" s="2"/>
+      <c r="F2" s="2" t="str">
+        <f>IF(ISNUMBER(D2),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G2" s="2">
+        <f>IF(ISNUMBER(D2),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H2" s="2" t="s">
         <v>239</v>
       </c>
@@ -6569,10 +6579,14 @@
         <f>D3/K3</f>
         <v>0.26272847570445024</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G3" s="2"/>
+      <c r="F3" s="2" t="str">
+        <f>IF(ISNUMBER(D3),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G3" s="2">
+        <f>IF(ISNUMBER(D3),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H3" s="2" t="s">
         <v>243</v>
       </c>
@@ -6616,10 +6630,14 @@
         <f>D4/K4</f>
         <v>0.1704064660696822</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G4" s="2"/>
+      <c r="F4" s="2" t="str">
+        <f>IF(ISNUMBER(D4),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G4" s="2">
+        <f>IF(ISNUMBER(D4),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H4" s="2" t="s">
         <v>247</v>
       </c>
@@ -6663,10 +6681,14 @@
         <f>D5/K5</f>
         <v>0.42178980296441965</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G5" s="2"/>
+      <c r="F5" s="2" t="str">
+        <f>IF(ISNUMBER(D5),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G5" s="2">
+        <f>IF(ISNUMBER(D5),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H5" s="2" t="s">
         <v>247</v>
       </c>
@@ -6710,10 +6732,14 @@
         <f>D6/K6</f>
         <v>0.3735385929393281</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G6" s="2"/>
+      <c r="F6" s="2" t="str">
+        <f>IF(ISNUMBER(D6),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G6" s="2">
+        <f>IF(ISNUMBER(D6),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H6" s="2" t="s">
         <v>247</v>
       </c>
@@ -6757,10 +6783,14 @@
         <f>D7/K7</f>
         <v>0.2508089498436376</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G7" s="2"/>
+      <c r="F7" s="2" t="str">
+        <f>IF(ISNUMBER(D7),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G7" s="2">
+        <f>IF(ISNUMBER(D7),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H7" s="2" t="s">
         <v>247</v>
       </c>
@@ -6804,10 +6834,14 @@
         <f>D8/K8</f>
         <v>0.0898816312523935</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G8" s="2"/>
+      <c r="F8" s="2" t="str">
+        <f>IF(ISNUMBER(D8),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G8" s="2">
+        <f>IF(ISNUMBER(D8),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H8" s="2" t="s">
         <v>247</v>
       </c>
@@ -6851,10 +6885,14 @@
         <f>D9/K9</f>
         <v>-0.23829318777202804</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G9" s="2"/>
+      <c r="F9" s="2" t="str">
+        <f>IF(ISNUMBER(D9),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G9" s="2">
+        <f>IF(ISNUMBER(D9),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H9" s="2" t="s">
         <v>247</v>
       </c>
@@ -6898,10 +6936,14 @@
         <f>D10/K10</f>
         <v>0.391578947368421</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G10" s="2"/>
+      <c r="F10" s="2" t="str">
+        <f>IF(ISNUMBER(D10),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G10" s="2">
+        <f>IF(ISNUMBER(D10),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H10" s="2" t="s">
         <v>247</v>
       </c>
@@ -6945,10 +6987,14 @@
         <f>D11/K11</f>
         <v>1.7349444677696384</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G11" s="2"/>
+      <c r="F11" s="2" t="str">
+        <f>IF(ISNUMBER(D11),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G11" s="2">
+        <f>IF(ISNUMBER(D11),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H11" s="2" t="s">
         <v>263</v>
       </c>
@@ -6992,10 +7038,14 @@
         <f>D12/K12</f>
         <v>133219980.0</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G12" s="2"/>
+      <c r="F12" s="2" t="str">
+        <f>IF(ISNUMBER(D12),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G12" s="2">
+        <f>IF(ISNUMBER(D12),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H12" s="2" t="s">
         <v>267</v>
       </c>
@@ -7039,10 +7089,14 @@
         <f>D13/K13</f>
         <v>33216205.0</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G13" s="2"/>
+      <c r="F13" s="2" t="str">
+        <f>IF(ISNUMBER(D13),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G13" s="2">
+        <f>IF(ISNUMBER(D13),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H13" s="2" t="s">
         <v>270</v>
       </c>
@@ -7086,10 +7140,14 @@
         <f>D14/K14</f>
         <v>90875424.0</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G14" s="2"/>
+      <c r="F14" s="2" t="str">
+        <f>IF(ISNUMBER(D14),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G14" s="2">
+        <f>IF(ISNUMBER(D14),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H14" s="2" t="s">
         <v>273</v>
       </c>
@@ -7133,10 +7191,14 @@
         <f>D15/K15</f>
         <v>29770009.0</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G15" s="2"/>
+      <c r="F15" s="2" t="str">
+        <f>IF(ISNUMBER(D15),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G15" s="2">
+        <f>IF(ISNUMBER(D15),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H15" s="2" t="s">
         <v>277</v>
       </c>
@@ -7180,10 +7242,14 @@
         <f>D16/K16</f>
         <v>299929743.0</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G16" s="2"/>
+      <c r="F16" s="2" t="str">
+        <f>IF(ISNUMBER(D16),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G16" s="2">
+        <f>IF(ISNUMBER(D16),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H16" s="2" t="s">
         <v>280</v>
       </c>
@@ -7227,10 +7293,14 @@
         <f>D17/K17</f>
         <v>974827544.0</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G17" s="2"/>
+      <c r="F17" s="2" t="str">
+        <f>IF(ISNUMBER(D17),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G17" s="2">
+        <f>IF(ISNUMBER(D17),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H17" s="2" t="s">
         <v>283</v>
       </c>
@@ -7272,10 +7342,14 @@
         <f>D18/K18</f>
         <v>76786309.0</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G18" s="2"/>
+      <c r="F18" s="2" t="str">
+        <f>IF(ISNUMBER(D18),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G18" s="2">
+        <f>IF(ISNUMBER(D18),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H18" s="2" t="s">
         <v>286</v>
       </c>
@@ -7319,10 +7393,14 @@
         <f>D19/K19</f>
         <v>371026323.0</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G19" s="2"/>
+      <c r="F19" s="2" t="str">
+        <f>IF(ISNUMBER(D19),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G19" s="2">
+        <f>IF(ISNUMBER(D19),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H19" s="2" t="s">
         <v>289</v>
       </c>
@@ -7366,10 +7444,14 @@
         <f>D20/K20</f>
         <v>119601197.0</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G20" s="2"/>
+      <c r="F20" s="2" t="str">
+        <f>IF(ISNUMBER(D20),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G20" s="2">
+        <f>IF(ISNUMBER(D20),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H20" s="2" t="s">
         <v>292</v>
       </c>
@@ -7413,10 +7495,14 @@
         <f>D21/K21</f>
         <v>37222781.0</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G21" s="2"/>
+      <c r="F21" s="2" t="str">
+        <f>IF(ISNUMBER(D21),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G21" s="2">
+        <f>IF(ISNUMBER(D21),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H21" s="2" t="s">
         <v>295</v>
       </c>
@@ -7458,10 +7544,14 @@
         <f>D22/K22</f>
         <v>-7139628.0</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G22" s="2"/>
+      <c r="F22" s="2" t="str">
+        <f>IF(ISNUMBER(D22),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G22" s="2">
+        <f>IF(ISNUMBER(D22),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H22" s="2" t="s">
         <v>298</v>
       </c>
@@ -7503,10 +7593,14 @@
         <f>D23/K23</f>
         <v>333512926.0</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G23" s="2"/>
+      <c r="F23" s="2" t="str">
+        <f>IF(ISNUMBER(D23),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G23" s="2">
+        <f>IF(ISNUMBER(D23),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H23" s="2" t="s">
         <v>301</v>
       </c>
@@ -7548,10 +7642,14 @@
         <f>D24/K24</f>
         <v>33583186.0</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G24" s="2"/>
+      <c r="F24" s="2" t="str">
+        <f>IF(ISNUMBER(D24),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G24" s="2">
+        <f>IF(ISNUMBER(D24),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H24" s="2" t="s">
         <v>304</v>
       </c>
@@ -7593,10 +7691,14 @@
         <f>D25/K25</f>
         <v>156823978.0</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G25" s="2"/>
+      <c r="F25" s="2" t="str">
+        <f>IF(ISNUMBER(D25),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G25" s="2">
+        <f>IF(ISNUMBER(D25),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H25" s="2" t="s">
         <v>307</v>
       </c>
@@ -7638,10 +7740,14 @@
         <f>D26/K26</f>
         <v>292018890.0</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G26" s="2"/>
+      <c r="F26" s="2" t="str">
+        <f>IF(ISNUMBER(D26),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G26" s="2">
+        <f>IF(ISNUMBER(D26),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H26" s="2" t="s">
         <v>311</v>
       </c>
@@ -7685,10 +7791,14 @@
         <f>D27/K27</f>
         <v>0.24724866942683058</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G27" s="2"/>
+      <c r="F27" s="2" t="str">
+        <f>IF(ISNUMBER(D27),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G27" s="2">
+        <f>IF(ISNUMBER(D27),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H27" s="2" t="s">
         <v>314</v>
       </c>
@@ -7732,10 +7842,14 @@
         <f>D28/K28</f>
         <v>2659992.0</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="G28" s="2"/>
+      <c r="F28" s="2" t="str">
+        <f>IF(ISNUMBER(D28),"calculated","not_calculated")</f>
+        <v>calculated</v>
+      </c>
+      <c r="G28" s="2">
+        <f>IF(ISNUMBER(D28),"","检查缺失值、分母与输入；口径变更须重跑Python")</f>
+        <v/>
+      </c>
       <c r="H28" s="2" t="s">
         <v>318</v>
       </c>
@@ -7767,13 +7881,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="8" width="28.7109375" customWidth="1"/>
+    <col min="1" max="9" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="32" customHeight="1">
+    <row r="1" spans="1:9" ht="32" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -7798,13 +7912,16 @@
       <c r="H1" s="1" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>281</v>
@@ -7819,19 +7936,24 @@
       <c r="F2" s="2">
         <v>0</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>355</v>
+      <c r="G2" s="2" t="str">
+        <f>IF(COUNT(E2,F2)&lt;2,"not_tested",IF(ABS(E2)&lt;=F2,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I2" s="2">
+        <f>IF(ISNUMBER(E2),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>284</v>
@@ -7846,19 +7968,24 @@
       <c r="F3" s="2">
         <v>1000</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>355</v>
+      <c r="G3" s="2" t="str">
+        <f>IF(COUNT(E3,F3)&lt;2,"not_tested",IF(ABS(E3)&lt;=F3,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I3" s="2">
+        <f>IF(ISNUMBER(E3),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>265</v>
@@ -7873,19 +8000,24 @@
       <c r="F4" s="2">
         <v>10000</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>355</v>
+      <c r="G4" s="2" t="str">
+        <f>IF(COUNT(E4,F4)&lt;2,"not_tested",IF(ABS(E4)&lt;=F4,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I4" s="2">
+        <f>IF(ISNUMBER(E4),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>275</v>
@@ -7900,19 +8032,24 @@
       <c r="F5" s="2">
         <v>2000</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>355</v>
+      <c r="G5" s="2" t="str">
+        <f>IF(COUNT(E5,F5)&lt;2,"not_tested",IF(ABS(E5)&lt;=F5,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I5" s="2">
+        <f>IF(ISNUMBER(E5),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>278</v>
@@ -7927,19 +8064,24 @@
       <c r="F6" s="2">
         <v>3000</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>355</v>
+      <c r="G6" s="2" t="str">
+        <f>IF(COUNT(E6,F6)&lt;2,"not_tested",IF(ABS(E6)&lt;=F6,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I6" s="2">
+        <f>IF(ISNUMBER(E6),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>287</v>
@@ -7954,19 +8096,24 @@
       <c r="F7" s="2">
         <v>3000</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>355</v>
+      <c r="G7" s="2" t="str">
+        <f>IF(COUNT(E7,F7)&lt;2,"not_tested",IF(ABS(E7)&lt;=F7,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I7" s="2">
+        <f>IF(ISNUMBER(E7),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>290</v>
@@ -7981,19 +8128,24 @@
       <c r="F8" s="2">
         <v>3000</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>355</v>
+      <c r="G8" s="2" t="str">
+        <f>IF(COUNT(E8,F8)&lt;2,"not_tested",IF(ABS(E8)&lt;=F8,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I8" s="2">
+        <f>IF(ISNUMBER(E8),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>293</v>
@@ -8008,19 +8160,24 @@
       <c r="F9" s="2">
         <v>1000</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>355</v>
+      <c r="G9" s="2" t="str">
+        <f>IF(COUNT(E9,F9)&lt;2,"not_tested",IF(ABS(E9)&lt;=F9,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I9" s="2">
+        <f>IF(ISNUMBER(E9),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>299</v>
@@ -8035,19 +8192,24 @@
       <c r="F10" s="2">
         <v>2000</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>355</v>
+      <c r="G10" s="2" t="str">
+        <f>IF(COUNT(E10,F10)&lt;2,"not_tested",IF(ABS(E10)&lt;=F10,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>357</v>
+      </c>
+      <c r="I10" s="2">
+        <f>IF(ISNUMBER(E10),"","missing or unavailable input")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>302</v>
@@ -8062,67 +8224,76 @@
       <c r="F11" s="2">
         <v>2000</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>355</v>
+      <c r="G11" s="2" t="str">
+        <f>IF(COUNT(E11,F11)&lt;2,"not_tested",IF(ABS(E11)&lt;=F11,"within_input_tolerance","unexplained_difference"))</f>
+        <v>within_input_tolerance</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
+      </c>
+      <c r="I11" s="2">
+        <f>IF(ISNUMBER(E11),"","missing or unavailable input")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:I11"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
     <col min="2" max="2" width="60.7109375" customWidth="1"/>
     <col min="3" max="3" width="100.7109375" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="70.7109375" customWidth="1"/>
+    <col min="5" max="6" width="70.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="32" customHeight="1">
+    <row r="1" spans="1:6" ht="32" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>379</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>382</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="F2" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:F2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -8143,16 +8314,16 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -8160,16 +8331,16 @@
         <v>118</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -8177,16 +8348,16 @@
         <v>74</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -8194,16 +8365,16 @@
         <v>40</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -8211,16 +8382,16 @@
         <v>63</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -8228,33 +8399,33 @@
         <v>145</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -8262,16 +8433,16 @@
         <v>58</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -8279,16 +8450,16 @@
         <v>113</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -8296,16 +8467,16 @@
         <v>103</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -8313,16 +8484,16 @@
         <v>68</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -8330,16 +8501,16 @@
         <v>160</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -8347,33 +8518,33 @@
         <v>108</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -8401,223 +8572,223 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>103</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>58</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>118</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
   </sheetData>
@@ -8639,93 +8810,93 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="2" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" s="2" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
   </sheetData>
@@ -8751,59 +8922,59 @@
         <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
   </sheetData>

</xml_diff>